<commit_message>
feat: Enhance MS signal creation with prefix detection and operator highlighting
- Implemented prefix-based signal type detection to clarify port references (i1, o1, p1, c1, r1).
- Updated logic to prevent plain numbers from being mapped to input ports, ensuring they remain as literals.
- Extended operator highlighting to cover all Verilog operators, improving syntax visibility in the TUI.
- Added comprehensive test suite for prefix detection and operator highlighting, ensuring all features function as intended.
- Documented changes and usage examples in MS_SIGNAL_ENHANCEMENTS.md for better user guidance.
</commit_message>
<xml_diff>
--- a/out/sessions/blur_scaler-20251110_152215/blur_scaler.xlsx
+++ b/out/sessions/blur_scaler-20251110_152215/blur_scaler.xlsx
@@ -1889,7 +1889,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="B1:N29"/>
+  <dimension ref="A1:N29"/>
   <sheetFormatPr baseColWidth="8" defaultColWidth="9" defaultRowHeight="13.5"/>
   <cols>
     <col width="9" customWidth="1" style="53" min="1" max="1"/>
@@ -2211,6 +2211,21 @@
           <t>1</t>
         </is>
       </c>
+      <c r="L11" s="92" t="inlineStr">
+        <is>
+          <t>new_val</t>
+        </is>
+      </c>
+      <c r="M11" s="92" t="inlineStr">
+        <is>
+          <t>i_blur_mode_cap + i_den +</t>
+        </is>
+      </c>
+      <c r="N11" s="92" t="inlineStr">
+        <is>
+          <t>3</t>
+        </is>
+      </c>
     </row>
     <row r="12">
       <c r="E12" s="92" t="inlineStr">
@@ -2241,6 +2256,21 @@
       <c r="J12" s="92" t="inlineStr">
         <is>
           <t>1</t>
+        </is>
+      </c>
+      <c r="L12" s="92" t="inlineStr">
+        <is>
+          <t>new</t>
+        </is>
+      </c>
+      <c r="M12" s="92" t="inlineStr">
+        <is>
+          <t>i_blur_mode_cap &amp;&amp; i_den &amp;&amp; i_hor_cnt &amp;&amp; i_hsync &amp;&amp;</t>
+        </is>
+      </c>
+      <c r="N12" s="92" t="inlineStr">
+        <is>
+          <t>6</t>
         </is>
       </c>
     </row>
@@ -7867,7 +7897,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A2:O39"/>
+  <dimension ref="B2:O39"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="13.5"/>
   <cols>
     <col width="4.375" customWidth="1" style="125" min="1" max="1"/>
@@ -8111,7 +8141,6 @@
       <c r="N21" s="128" t="n"/>
       <c r="O21" s="129" t="n"/>
     </row>
-    <row r="22"/>
     <row r="23" ht="26.25" customHeight="1" s="125">
       <c r="I23" s="116" t="n"/>
       <c r="J23" s="117" t="n"/>

</xml_diff>